<commit_message>
Add network schedule (Гантт-стиль) sheet to workbook
Co-authored-by: boldashevalexandr-eng <boldashevalexandr-eng@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/Основной_график_18053-ТУ_лот2.xlsx
+++ b/output/Основной_график_18053-ТУ_лот2.xlsx
@@ -7,10 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Основной график" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Сетевой график" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Основной график" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Основной график'!$1:$2</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Сетевой график'!$1:$3</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Основной график'!$1:$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -51,8 +53,33 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -74,8 +101,38 @@
         <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E75B6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C00000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF5EC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="005B9BD5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F5F7FA"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -97,11 +154,83 @@
         <color rgb="00808080"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00808080"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00808080"/>
+      </right>
+      <top style="thin">
+        <color rgb="00808080"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00808080"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00808080"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00808080"/>
+      </right>
+      <top style="thin">
+        <color rgb="00808080"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00808080"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="009AA0A6"/>
+      </left>
+      <right style="thin">
+        <color rgb="009AA0A6"/>
+      </right>
+      <top style="thin">
+        <color rgb="009AA0A6"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="009AA0A6"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="hair">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="hair">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="hair">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="hair">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -137,6 +266,64 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -502,6 +689,1529 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
+  <dimension ref="A1:AR20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="6" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="4" customWidth="1" min="10" max="10"/>
+    <col width="4" customWidth="1" min="11" max="11"/>
+    <col width="4" customWidth="1" min="12" max="12"/>
+    <col width="4" customWidth="1" min="13" max="13"/>
+    <col width="4" customWidth="1" min="14" max="14"/>
+    <col width="4" customWidth="1" min="15" max="15"/>
+    <col width="4" customWidth="1" min="16" max="16"/>
+    <col width="4" customWidth="1" min="17" max="17"/>
+    <col width="4" customWidth="1" min="18" max="18"/>
+    <col width="4" customWidth="1" min="19" max="19"/>
+    <col width="4" customWidth="1" min="20" max="20"/>
+    <col width="4" customWidth="1" min="21" max="21"/>
+    <col width="4" customWidth="1" min="22" max="22"/>
+    <col width="4" customWidth="1" min="23" max="23"/>
+    <col width="4" customWidth="1" min="24" max="24"/>
+    <col width="4" customWidth="1" min="25" max="25"/>
+    <col width="4" customWidth="1" min="26" max="26"/>
+    <col width="4" customWidth="1" min="27" max="27"/>
+    <col width="4" customWidth="1" min="28" max="28"/>
+    <col width="4" customWidth="1" min="29" max="29"/>
+    <col width="4" customWidth="1" min="30" max="30"/>
+    <col width="4" customWidth="1" min="31" max="31"/>
+    <col width="4" customWidth="1" min="32" max="32"/>
+    <col width="4" customWidth="1" min="33" max="33"/>
+    <col width="4" customWidth="1" min="34" max="34"/>
+    <col width="4" customWidth="1" min="35" max="35"/>
+    <col width="4" customWidth="1" min="36" max="36"/>
+    <col width="4" customWidth="1" min="37" max="37"/>
+    <col width="4" customWidth="1" min="38" max="38"/>
+    <col width="4" customWidth="1" min="39" max="39"/>
+    <col width="4" customWidth="1" min="40" max="40"/>
+    <col width="4" customWidth="1" min="41" max="41"/>
+    <col width="4" customWidth="1" min="42" max="42"/>
+    <col width="4" customWidth="1" min="43" max="43"/>
+    <col width="4" customWidth="1" min="44" max="44"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="60" customHeight="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>СЕТЕВОЙ (КАЛЕНДАРНО-СЕТЕВОЙ) ГРАФИК ПРОИЗВОДСТВА РАБОТ
+Объект: Магистральный трубопровод из труб ПНД (DN 50 – DN 500). Лот №2, шифр 18053-ТУ.   Подрядчик: ООО «МАГУС-СТРОЙ»
+Начало: 27.06.2026    Окончание: 21.02.2027    Срок: 240 календ. дней    ★ — критический путь</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="14" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B2" s="14" t="inlineStr">
+        <is>
+          <t>Шифр</t>
+        </is>
+      </c>
+      <c r="C2" s="14" t="inlineStr">
+        <is>
+          <t>Работа</t>
+        </is>
+      </c>
+      <c r="D2" s="14" t="inlineStr">
+        <is>
+          <t>Предш.</t>
+        </is>
+      </c>
+      <c r="E2" s="14" t="inlineStr">
+        <is>
+          <t>Бригада</t>
+        </is>
+      </c>
+      <c r="F2" s="14" t="inlineStr">
+        <is>
+          <t>Начало</t>
+        </is>
+      </c>
+      <c r="G2" s="14" t="inlineStr">
+        <is>
+          <t>Окончание</t>
+        </is>
+      </c>
+      <c r="H2" s="14" t="inlineStr">
+        <is>
+          <t>Дней</t>
+        </is>
+      </c>
+      <c r="I2" s="14" t="inlineStr">
+        <is>
+          <t>Резерв, дн.</t>
+        </is>
+      </c>
+      <c r="J2" s="15" t="inlineStr">
+        <is>
+          <t>ИЮНЬ 2026</t>
+        </is>
+      </c>
+      <c r="K2" s="15" t="inlineStr">
+        <is>
+          <t>ИЮЛЬ 2026</t>
+        </is>
+      </c>
+      <c r="O2" s="15" t="inlineStr">
+        <is>
+          <t>АВГУСТ 2026</t>
+        </is>
+      </c>
+      <c r="T2" s="15" t="inlineStr">
+        <is>
+          <t>СЕНТЯБРЬ 2026</t>
+        </is>
+      </c>
+      <c r="X2" s="15" t="inlineStr">
+        <is>
+          <t>ОКТЯБРЬ 2026</t>
+        </is>
+      </c>
+      <c r="AC2" s="15" t="inlineStr">
+        <is>
+          <t>НОЯБРЬ 2026</t>
+        </is>
+      </c>
+      <c r="AG2" s="15" t="inlineStr">
+        <is>
+          <t>ДЕКАБРЬ 2026</t>
+        </is>
+      </c>
+      <c r="AK2" s="15" t="inlineStr">
+        <is>
+          <t>ЯНВАРЬ 2027</t>
+        </is>
+      </c>
+      <c r="AP2" s="15" t="inlineStr">
+        <is>
+          <t>ФЕВРАЛЬ 2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="J3" s="16" t="inlineStr">
+        <is>
+          <t>27.06</t>
+        </is>
+      </c>
+      <c r="K3" s="16" t="inlineStr">
+        <is>
+          <t>04.07</t>
+        </is>
+      </c>
+      <c r="L3" s="16" t="inlineStr">
+        <is>
+          <t>11.07</t>
+        </is>
+      </c>
+      <c r="M3" s="16" t="inlineStr">
+        <is>
+          <t>18.07</t>
+        </is>
+      </c>
+      <c r="N3" s="16" t="inlineStr">
+        <is>
+          <t>25.07</t>
+        </is>
+      </c>
+      <c r="O3" s="16" t="inlineStr">
+        <is>
+          <t>01.08</t>
+        </is>
+      </c>
+      <c r="P3" s="16" t="inlineStr">
+        <is>
+          <t>08.08</t>
+        </is>
+      </c>
+      <c r="Q3" s="16" t="inlineStr">
+        <is>
+          <t>15.08</t>
+        </is>
+      </c>
+      <c r="R3" s="16" t="inlineStr">
+        <is>
+          <t>22.08</t>
+        </is>
+      </c>
+      <c r="S3" s="16" t="inlineStr">
+        <is>
+          <t>29.08</t>
+        </is>
+      </c>
+      <c r="T3" s="16" t="inlineStr">
+        <is>
+          <t>05.09</t>
+        </is>
+      </c>
+      <c r="U3" s="16" t="inlineStr">
+        <is>
+          <t>12.09</t>
+        </is>
+      </c>
+      <c r="V3" s="16" t="inlineStr">
+        <is>
+          <t>19.09</t>
+        </is>
+      </c>
+      <c r="W3" s="16" t="inlineStr">
+        <is>
+          <t>26.09</t>
+        </is>
+      </c>
+      <c r="X3" s="16" t="inlineStr">
+        <is>
+          <t>03.10</t>
+        </is>
+      </c>
+      <c r="Y3" s="16" t="inlineStr">
+        <is>
+          <t>10.10</t>
+        </is>
+      </c>
+      <c r="Z3" s="16" t="inlineStr">
+        <is>
+          <t>17.10</t>
+        </is>
+      </c>
+      <c r="AA3" s="16" t="inlineStr">
+        <is>
+          <t>24.10</t>
+        </is>
+      </c>
+      <c r="AB3" s="16" t="inlineStr">
+        <is>
+          <t>31.10</t>
+        </is>
+      </c>
+      <c r="AC3" s="16" t="inlineStr">
+        <is>
+          <t>07.11</t>
+        </is>
+      </c>
+      <c r="AD3" s="16" t="inlineStr">
+        <is>
+          <t>14.11</t>
+        </is>
+      </c>
+      <c r="AE3" s="16" t="inlineStr">
+        <is>
+          <t>21.11</t>
+        </is>
+      </c>
+      <c r="AF3" s="16" t="inlineStr">
+        <is>
+          <t>28.11</t>
+        </is>
+      </c>
+      <c r="AG3" s="16" t="inlineStr">
+        <is>
+          <t>05.12</t>
+        </is>
+      </c>
+      <c r="AH3" s="16" t="inlineStr">
+        <is>
+          <t>12.12</t>
+        </is>
+      </c>
+      <c r="AI3" s="16" t="inlineStr">
+        <is>
+          <t>19.12</t>
+        </is>
+      </c>
+      <c r="AJ3" s="16" t="inlineStr">
+        <is>
+          <t>26.12</t>
+        </is>
+      </c>
+      <c r="AK3" s="16" t="inlineStr">
+        <is>
+          <t>02.01</t>
+        </is>
+      </c>
+      <c r="AL3" s="16" t="inlineStr">
+        <is>
+          <t>09.01</t>
+        </is>
+      </c>
+      <c r="AM3" s="16" t="inlineStr">
+        <is>
+          <t>16.01</t>
+        </is>
+      </c>
+      <c r="AN3" s="16" t="inlineStr">
+        <is>
+          <t>23.01</t>
+        </is>
+      </c>
+      <c r="AO3" s="16" t="inlineStr">
+        <is>
+          <t>30.01</t>
+        </is>
+      </c>
+      <c r="AP3" s="16" t="inlineStr">
+        <is>
+          <t>06.02</t>
+        </is>
+      </c>
+      <c r="AQ3" s="16" t="inlineStr">
+        <is>
+          <t>13.02</t>
+        </is>
+      </c>
+      <c r="AR3" s="16" t="inlineStr">
+        <is>
+          <t>20.02</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="36" customHeight="1">
+      <c r="A4" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C4" s="18" t="inlineStr">
+        <is>
+          <t>Подготовительные и орг.-техн. работы (мобилизация, бытовка, ограждение)</t>
+        </is>
+      </c>
+      <c r="D4" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E4" s="19" t="inlineStr">
+        <is>
+          <t>Бр.№1 подгот.</t>
+        </is>
+      </c>
+      <c r="F4" s="17" t="inlineStr">
+        <is>
+          <t>27.06.2026</t>
+        </is>
+      </c>
+      <c r="G4" s="17" t="inlineStr">
+        <is>
+          <t>11.07.2026</t>
+        </is>
+      </c>
+      <c r="H4" s="17" t="n">
+        <v>15</v>
+      </c>
+      <c r="I4" s="17" t="inlineStr">
+        <is>
+          <t>0 ★</t>
+        </is>
+      </c>
+      <c r="J4" s="20" t="inlineStr">
+        <is>
+          <t>★1</t>
+        </is>
+      </c>
+      <c r="K4" s="21" t="n"/>
+      <c r="L4" s="21" t="n"/>
+      <c r="M4" s="22" t="n"/>
+      <c r="N4" s="22" t="n"/>
+      <c r="O4" s="22" t="n"/>
+      <c r="P4" s="22" t="n"/>
+      <c r="Q4" s="22" t="n"/>
+      <c r="R4" s="22" t="n"/>
+      <c r="S4" s="22" t="n"/>
+      <c r="T4" s="22" t="n"/>
+      <c r="U4" s="22" t="n"/>
+      <c r="V4" s="22" t="n"/>
+      <c r="W4" s="22" t="n"/>
+      <c r="X4" s="22" t="n"/>
+      <c r="Y4" s="22" t="n"/>
+      <c r="Z4" s="22" t="n"/>
+      <c r="AA4" s="22" t="n"/>
+      <c r="AB4" s="22" t="n"/>
+      <c r="AC4" s="22" t="n"/>
+      <c r="AD4" s="22" t="n"/>
+      <c r="AE4" s="22" t="n"/>
+      <c r="AF4" s="22" t="n"/>
+      <c r="AG4" s="22" t="n"/>
+      <c r="AH4" s="22" t="n"/>
+      <c r="AI4" s="22" t="n"/>
+      <c r="AJ4" s="22" t="n"/>
+      <c r="AK4" s="22" t="n"/>
+      <c r="AL4" s="22" t="n"/>
+      <c r="AM4" s="22" t="n"/>
+      <c r="AN4" s="22" t="n"/>
+      <c r="AO4" s="22" t="n"/>
+      <c r="AP4" s="22" t="n"/>
+      <c r="AQ4" s="22" t="n"/>
+      <c r="AR4" s="22" t="n"/>
+    </row>
+    <row r="5" ht="36" customHeight="1">
+      <c r="A5" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="17" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C5" s="18" t="inlineStr">
+        <is>
+          <t>Геодезическая разбивка трассы, вынос осей и реперов</t>
+        </is>
+      </c>
+      <c r="D5" s="19" t="inlineStr">
+        <is>
+          <t>1(НН+9)</t>
+        </is>
+      </c>
+      <c r="E5" s="19" t="inlineStr">
+        <is>
+          <t>Геодез. гр.</t>
+        </is>
+      </c>
+      <c r="F5" s="17" t="inlineStr">
+        <is>
+          <t>06.07.2026</t>
+        </is>
+      </c>
+      <c r="G5" s="17" t="inlineStr">
+        <is>
+          <t>15.07.2026</t>
+        </is>
+      </c>
+      <c r="H5" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="I5" s="17" t="inlineStr">
+        <is>
+          <t>0 ★</t>
+        </is>
+      </c>
+      <c r="J5" s="22" t="n"/>
+      <c r="K5" s="20" t="inlineStr">
+        <is>
+          <t>★2</t>
+        </is>
+      </c>
+      <c r="L5" s="21" t="n"/>
+      <c r="M5" s="22" t="n"/>
+      <c r="N5" s="22" t="n"/>
+      <c r="O5" s="22" t="n"/>
+      <c r="P5" s="22" t="n"/>
+      <c r="Q5" s="22" t="n"/>
+      <c r="R5" s="22" t="n"/>
+      <c r="S5" s="22" t="n"/>
+      <c r="T5" s="22" t="n"/>
+      <c r="U5" s="22" t="n"/>
+      <c r="V5" s="22" t="n"/>
+      <c r="W5" s="22" t="n"/>
+      <c r="X5" s="22" t="n"/>
+      <c r="Y5" s="22" t="n"/>
+      <c r="Z5" s="22" t="n"/>
+      <c r="AA5" s="22" t="n"/>
+      <c r="AB5" s="22" t="n"/>
+      <c r="AC5" s="22" t="n"/>
+      <c r="AD5" s="22" t="n"/>
+      <c r="AE5" s="22" t="n"/>
+      <c r="AF5" s="22" t="n"/>
+      <c r="AG5" s="22" t="n"/>
+      <c r="AH5" s="22" t="n"/>
+      <c r="AI5" s="22" t="n"/>
+      <c r="AJ5" s="22" t="n"/>
+      <c r="AK5" s="22" t="n"/>
+      <c r="AL5" s="22" t="n"/>
+      <c r="AM5" s="22" t="n"/>
+      <c r="AN5" s="22" t="n"/>
+      <c r="AO5" s="22" t="n"/>
+      <c r="AP5" s="22" t="n"/>
+      <c r="AQ5" s="22" t="n"/>
+      <c r="AR5" s="22" t="n"/>
+    </row>
+    <row r="6" ht="36" customHeight="1">
+      <c r="A6" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="17" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>Земляные работы: разработка траншеи DN 50 – DN 500, песчаная подготовка</t>
+        </is>
+      </c>
+      <c r="D6" s="19" t="inlineStr">
+        <is>
+          <t>1; 2(НН+6)</t>
+        </is>
+      </c>
+      <c r="E6" s="19" t="inlineStr">
+        <is>
+          <t>Бр.№2 земл.</t>
+        </is>
+      </c>
+      <c r="F6" s="17" t="inlineStr">
+        <is>
+          <t>12.07.2026</t>
+        </is>
+      </c>
+      <c r="G6" s="17" t="inlineStr">
+        <is>
+          <t>14.10.2026</t>
+        </is>
+      </c>
+      <c r="H6" s="17" t="n">
+        <v>95</v>
+      </c>
+      <c r="I6" s="17" t="inlineStr">
+        <is>
+          <t>0 ★</t>
+        </is>
+      </c>
+      <c r="J6" s="22" t="n"/>
+      <c r="K6" s="22" t="n"/>
+      <c r="L6" s="20" t="inlineStr">
+        <is>
+          <t>★3</t>
+        </is>
+      </c>
+      <c r="M6" s="21" t="n"/>
+      <c r="N6" s="21" t="n"/>
+      <c r="O6" s="21" t="n"/>
+      <c r="P6" s="21" t="n"/>
+      <c r="Q6" s="21" t="n"/>
+      <c r="R6" s="21" t="n"/>
+      <c r="S6" s="21" t="n"/>
+      <c r="T6" s="21" t="n"/>
+      <c r="U6" s="21" t="n"/>
+      <c r="V6" s="21" t="n"/>
+      <c r="W6" s="21" t="n"/>
+      <c r="X6" s="21" t="n"/>
+      <c r="Y6" s="21" t="n"/>
+      <c r="Z6" s="22" t="n"/>
+      <c r="AA6" s="22" t="n"/>
+      <c r="AB6" s="22" t="n"/>
+      <c r="AC6" s="22" t="n"/>
+      <c r="AD6" s="22" t="n"/>
+      <c r="AE6" s="22" t="n"/>
+      <c r="AF6" s="22" t="n"/>
+      <c r="AG6" s="22" t="n"/>
+      <c r="AH6" s="22" t="n"/>
+      <c r="AI6" s="22" t="n"/>
+      <c r="AJ6" s="22" t="n"/>
+      <c r="AK6" s="22" t="n"/>
+      <c r="AL6" s="22" t="n"/>
+      <c r="AM6" s="22" t="n"/>
+      <c r="AN6" s="22" t="n"/>
+      <c r="AO6" s="22" t="n"/>
+      <c r="AP6" s="22" t="n"/>
+      <c r="AQ6" s="22" t="n"/>
+      <c r="AR6" s="22" t="n"/>
+    </row>
+    <row r="7" ht="36" customHeight="1">
+      <c r="A7" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C7" s="18" t="inlineStr">
+        <is>
+          <t>Монтаж магистрали ПНД SDR17 DN 500 — сварка встык, укладка</t>
+        </is>
+      </c>
+      <c r="D7" s="19" t="inlineStr">
+        <is>
+          <t>3(НН+15)</t>
+        </is>
+      </c>
+      <c r="E7" s="19" t="inlineStr">
+        <is>
+          <t>Бр.№3 монт.</t>
+        </is>
+      </c>
+      <c r="F7" s="17" t="inlineStr">
+        <is>
+          <t>27.07.2026</t>
+        </is>
+      </c>
+      <c r="G7" s="17" t="inlineStr">
+        <is>
+          <t>08.12.2026</t>
+        </is>
+      </c>
+      <c r="H7" s="17" t="n">
+        <v>135</v>
+      </c>
+      <c r="I7" s="17" t="inlineStr">
+        <is>
+          <t>0 ★</t>
+        </is>
+      </c>
+      <c r="J7" s="22" t="n"/>
+      <c r="K7" s="22" t="n"/>
+      <c r="L7" s="22" t="n"/>
+      <c r="M7" s="22" t="n"/>
+      <c r="N7" s="20" t="inlineStr">
+        <is>
+          <t>★4</t>
+        </is>
+      </c>
+      <c r="O7" s="21" t="n"/>
+      <c r="P7" s="21" t="n"/>
+      <c r="Q7" s="21" t="n"/>
+      <c r="R7" s="21" t="n"/>
+      <c r="S7" s="21" t="n"/>
+      <c r="T7" s="21" t="n"/>
+      <c r="U7" s="21" t="n"/>
+      <c r="V7" s="21" t="n"/>
+      <c r="W7" s="21" t="n"/>
+      <c r="X7" s="21" t="n"/>
+      <c r="Y7" s="21" t="n"/>
+      <c r="Z7" s="21" t="n"/>
+      <c r="AA7" s="21" t="n"/>
+      <c r="AB7" s="21" t="n"/>
+      <c r="AC7" s="21" t="n"/>
+      <c r="AD7" s="21" t="n"/>
+      <c r="AE7" s="21" t="n"/>
+      <c r="AF7" s="21" t="n"/>
+      <c r="AG7" s="21" t="n"/>
+      <c r="AH7" s="22" t="n"/>
+      <c r="AI7" s="22" t="n"/>
+      <c r="AJ7" s="22" t="n"/>
+      <c r="AK7" s="22" t="n"/>
+      <c r="AL7" s="22" t="n"/>
+      <c r="AM7" s="22" t="n"/>
+      <c r="AN7" s="22" t="n"/>
+      <c r="AO7" s="22" t="n"/>
+      <c r="AP7" s="22" t="n"/>
+      <c r="AQ7" s="22" t="n"/>
+      <c r="AR7" s="22" t="n"/>
+    </row>
+    <row r="8" ht="36" customHeight="1">
+      <c r="A8" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>Монтаж отводов ПНД DN 50 / DN 100 (электромуфты, врезки)</t>
+        </is>
+      </c>
+      <c r="D8" s="19" t="inlineStr">
+        <is>
+          <t>4(НН+55)</t>
+        </is>
+      </c>
+      <c r="E8" s="19" t="inlineStr">
+        <is>
+          <t>Бр.№3а монт.</t>
+        </is>
+      </c>
+      <c r="F8" s="17" t="inlineStr">
+        <is>
+          <t>20.09.2026</t>
+        </is>
+      </c>
+      <c r="G8" s="17" t="inlineStr">
+        <is>
+          <t>23.12.2026</t>
+        </is>
+      </c>
+      <c r="H8" s="17" t="n">
+        <v>95</v>
+      </c>
+      <c r="I8" s="17" t="inlineStr">
+        <is>
+          <t>0 ★</t>
+        </is>
+      </c>
+      <c r="J8" s="22" t="n"/>
+      <c r="K8" s="22" t="n"/>
+      <c r="L8" s="22" t="n"/>
+      <c r="M8" s="22" t="n"/>
+      <c r="N8" s="22" t="n"/>
+      <c r="O8" s="22" t="n"/>
+      <c r="P8" s="22" t="n"/>
+      <c r="Q8" s="22" t="n"/>
+      <c r="R8" s="22" t="n"/>
+      <c r="S8" s="22" t="n"/>
+      <c r="T8" s="22" t="n"/>
+      <c r="U8" s="22" t="n"/>
+      <c r="V8" s="20" t="inlineStr">
+        <is>
+          <t>★5</t>
+        </is>
+      </c>
+      <c r="W8" s="21" t="n"/>
+      <c r="X8" s="21" t="n"/>
+      <c r="Y8" s="21" t="n"/>
+      <c r="Z8" s="21" t="n"/>
+      <c r="AA8" s="21" t="n"/>
+      <c r="AB8" s="21" t="n"/>
+      <c r="AC8" s="21" t="n"/>
+      <c r="AD8" s="21" t="n"/>
+      <c r="AE8" s="21" t="n"/>
+      <c r="AF8" s="21" t="n"/>
+      <c r="AG8" s="21" t="n"/>
+      <c r="AH8" s="21" t="n"/>
+      <c r="AI8" s="21" t="n"/>
+      <c r="AJ8" s="22" t="n"/>
+      <c r="AK8" s="22" t="n"/>
+      <c r="AL8" s="22" t="n"/>
+      <c r="AM8" s="22" t="n"/>
+      <c r="AN8" s="22" t="n"/>
+      <c r="AO8" s="22" t="n"/>
+      <c r="AP8" s="22" t="n"/>
+      <c r="AQ8" s="22" t="n"/>
+      <c r="AR8" s="22" t="n"/>
+    </row>
+    <row r="9" ht="36" customHeight="1">
+      <c r="A9" s="23" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="23" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C9" s="24" t="inlineStr">
+        <is>
+          <t>Устройство смотровых / поворотных колодцев (ж/б сборные)</t>
+        </is>
+      </c>
+      <c r="D9" s="24" t="inlineStr">
+        <is>
+          <t>3(НН+45)</t>
+        </is>
+      </c>
+      <c r="E9" s="24" t="inlineStr">
+        <is>
+          <t>Бр.№4 кол.</t>
+        </is>
+      </c>
+      <c r="F9" s="23" t="inlineStr">
+        <is>
+          <t>26.08.2026</t>
+        </is>
+      </c>
+      <c r="G9" s="23" t="inlineStr">
+        <is>
+          <t>23.11.2026</t>
+        </is>
+      </c>
+      <c r="H9" s="23" t="n">
+        <v>90</v>
+      </c>
+      <c r="I9" s="23" t="n">
+        <v>90</v>
+      </c>
+      <c r="J9" s="25" t="n"/>
+      <c r="K9" s="25" t="n"/>
+      <c r="L9" s="25" t="n"/>
+      <c r="M9" s="25" t="n"/>
+      <c r="N9" s="25" t="n"/>
+      <c r="O9" s="25" t="n"/>
+      <c r="P9" s="25" t="n"/>
+      <c r="Q9" s="25" t="n"/>
+      <c r="R9" s="26" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="S9" s="27" t="n"/>
+      <c r="T9" s="27" t="n"/>
+      <c r="U9" s="27" t="n"/>
+      <c r="V9" s="27" t="n"/>
+      <c r="W9" s="27" t="n"/>
+      <c r="X9" s="27" t="n"/>
+      <c r="Y9" s="27" t="n"/>
+      <c r="Z9" s="27" t="n"/>
+      <c r="AA9" s="27" t="n"/>
+      <c r="AB9" s="27" t="n"/>
+      <c r="AC9" s="27" t="n"/>
+      <c r="AD9" s="27" t="n"/>
+      <c r="AE9" s="27" t="n"/>
+      <c r="AF9" s="25" t="n"/>
+      <c r="AG9" s="25" t="n"/>
+      <c r="AH9" s="25" t="n"/>
+      <c r="AI9" s="25" t="n"/>
+      <c r="AJ9" s="25" t="n"/>
+      <c r="AK9" s="25" t="n"/>
+      <c r="AL9" s="25" t="n"/>
+      <c r="AM9" s="25" t="n"/>
+      <c r="AN9" s="25" t="n"/>
+      <c r="AO9" s="25" t="n"/>
+      <c r="AP9" s="25" t="n"/>
+      <c r="AQ9" s="25" t="n"/>
+      <c r="AR9" s="25" t="n"/>
+    </row>
+    <row r="10" ht="36" customHeight="1">
+      <c r="A10" s="28" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="28" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C10" s="29" t="inlineStr">
+        <is>
+          <t>Установка запорной арматуры, фасонных изделий, ковров</t>
+        </is>
+      </c>
+      <c r="D10" s="29" t="inlineStr">
+        <is>
+          <t>4(НН+90)</t>
+        </is>
+      </c>
+      <c r="E10" s="29" t="inlineStr">
+        <is>
+          <t>Бр.№3б арм.</t>
+        </is>
+      </c>
+      <c r="F10" s="28" t="inlineStr">
+        <is>
+          <t>25.10.2026</t>
+        </is>
+      </c>
+      <c r="G10" s="28" t="inlineStr">
+        <is>
+          <t>02.01.2027</t>
+        </is>
+      </c>
+      <c r="H10" s="28" t="n">
+        <v>70</v>
+      </c>
+      <c r="I10" s="28" t="n">
+        <v>50</v>
+      </c>
+      <c r="J10" s="30" t="n"/>
+      <c r="K10" s="30" t="n"/>
+      <c r="L10" s="30" t="n"/>
+      <c r="M10" s="30" t="n"/>
+      <c r="N10" s="30" t="n"/>
+      <c r="O10" s="30" t="n"/>
+      <c r="P10" s="30" t="n"/>
+      <c r="Q10" s="30" t="n"/>
+      <c r="R10" s="30" t="n"/>
+      <c r="S10" s="30" t="n"/>
+      <c r="T10" s="30" t="n"/>
+      <c r="U10" s="30" t="n"/>
+      <c r="V10" s="30" t="n"/>
+      <c r="W10" s="30" t="n"/>
+      <c r="X10" s="30" t="n"/>
+      <c r="Y10" s="30" t="n"/>
+      <c r="Z10" s="30" t="n"/>
+      <c r="AA10" s="26" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="AB10" s="27" t="n"/>
+      <c r="AC10" s="27" t="n"/>
+      <c r="AD10" s="27" t="n"/>
+      <c r="AE10" s="27" t="n"/>
+      <c r="AF10" s="27" t="n"/>
+      <c r="AG10" s="27" t="n"/>
+      <c r="AH10" s="27" t="n"/>
+      <c r="AI10" s="27" t="n"/>
+      <c r="AJ10" s="27" t="n"/>
+      <c r="AK10" s="27" t="n"/>
+      <c r="AL10" s="30" t="n"/>
+      <c r="AM10" s="30" t="n"/>
+      <c r="AN10" s="30" t="n"/>
+      <c r="AO10" s="30" t="n"/>
+      <c r="AP10" s="30" t="n"/>
+      <c r="AQ10" s="30" t="n"/>
+      <c r="AR10" s="30" t="n"/>
+    </row>
+    <row r="11" ht="36" customHeight="1">
+      <c r="A11" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="23" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C11" s="24" t="inlineStr">
+        <is>
+          <t>Переходы через коммуникации и автодороги (ГНБ, футляры)</t>
+        </is>
+      </c>
+      <c r="D11" s="24" t="inlineStr">
+        <is>
+          <t>3(НН+55)</t>
+        </is>
+      </c>
+      <c r="E11" s="24" t="inlineStr">
+        <is>
+          <t>Бр.№5 ГНБ</t>
+        </is>
+      </c>
+      <c r="F11" s="23" t="inlineStr">
+        <is>
+          <t>05.09.2026</t>
+        </is>
+      </c>
+      <c r="G11" s="23" t="inlineStr">
+        <is>
+          <t>03.11.2026</t>
+        </is>
+      </c>
+      <c r="H11" s="23" t="n">
+        <v>60</v>
+      </c>
+      <c r="I11" s="23" t="n">
+        <v>110</v>
+      </c>
+      <c r="J11" s="25" t="n"/>
+      <c r="K11" s="25" t="n"/>
+      <c r="L11" s="25" t="n"/>
+      <c r="M11" s="25" t="n"/>
+      <c r="N11" s="25" t="n"/>
+      <c r="O11" s="25" t="n"/>
+      <c r="P11" s="25" t="n"/>
+      <c r="Q11" s="25" t="n"/>
+      <c r="R11" s="25" t="n"/>
+      <c r="S11" s="25" t="n"/>
+      <c r="T11" s="26" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="U11" s="27" t="n"/>
+      <c r="V11" s="27" t="n"/>
+      <c r="W11" s="27" t="n"/>
+      <c r="X11" s="27" t="n"/>
+      <c r="Y11" s="27" t="n"/>
+      <c r="Z11" s="27" t="n"/>
+      <c r="AA11" s="27" t="n"/>
+      <c r="AB11" s="27" t="n"/>
+      <c r="AC11" s="25" t="n"/>
+      <c r="AD11" s="25" t="n"/>
+      <c r="AE11" s="25" t="n"/>
+      <c r="AF11" s="25" t="n"/>
+      <c r="AG11" s="25" t="n"/>
+      <c r="AH11" s="25" t="n"/>
+      <c r="AI11" s="25" t="n"/>
+      <c r="AJ11" s="25" t="n"/>
+      <c r="AK11" s="25" t="n"/>
+      <c r="AL11" s="25" t="n"/>
+      <c r="AM11" s="25" t="n"/>
+      <c r="AN11" s="25" t="n"/>
+      <c r="AO11" s="25" t="n"/>
+      <c r="AP11" s="25" t="n"/>
+      <c r="AQ11" s="25" t="n"/>
+      <c r="AR11" s="25" t="n"/>
+    </row>
+    <row r="12" ht="36" customHeight="1">
+      <c r="A12" s="28" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" s="28" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C12" s="29" t="inlineStr">
+        <is>
+          <t>Контроль сварных стыков (ВИК, УЗК/рентген), ЭХЗ</t>
+        </is>
+      </c>
+      <c r="D12" s="29" t="inlineStr">
+        <is>
+          <t>4(НН+100)</t>
+        </is>
+      </c>
+      <c r="E12" s="29" t="inlineStr">
+        <is>
+          <t>Лаб. НК</t>
+        </is>
+      </c>
+      <c r="F12" s="28" t="inlineStr">
+        <is>
+          <t>04.11.2026</t>
+        </is>
+      </c>
+      <c r="G12" s="28" t="inlineStr">
+        <is>
+          <t>02.01.2027</t>
+        </is>
+      </c>
+      <c r="H12" s="28" t="n">
+        <v>60</v>
+      </c>
+      <c r="I12" s="28" t="n">
+        <v>50</v>
+      </c>
+      <c r="J12" s="30" t="n"/>
+      <c r="K12" s="30" t="n"/>
+      <c r="L12" s="30" t="n"/>
+      <c r="M12" s="30" t="n"/>
+      <c r="N12" s="30" t="n"/>
+      <c r="O12" s="30" t="n"/>
+      <c r="P12" s="30" t="n"/>
+      <c r="Q12" s="30" t="n"/>
+      <c r="R12" s="30" t="n"/>
+      <c r="S12" s="30" t="n"/>
+      <c r="T12" s="30" t="n"/>
+      <c r="U12" s="30" t="n"/>
+      <c r="V12" s="30" t="n"/>
+      <c r="W12" s="30" t="n"/>
+      <c r="X12" s="30" t="n"/>
+      <c r="Y12" s="30" t="n"/>
+      <c r="Z12" s="30" t="n"/>
+      <c r="AA12" s="30" t="n"/>
+      <c r="AB12" s="26" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="AC12" s="27" t="n"/>
+      <c r="AD12" s="27" t="n"/>
+      <c r="AE12" s="27" t="n"/>
+      <c r="AF12" s="27" t="n"/>
+      <c r="AG12" s="27" t="n"/>
+      <c r="AH12" s="27" t="n"/>
+      <c r="AI12" s="27" t="n"/>
+      <c r="AJ12" s="27" t="n"/>
+      <c r="AK12" s="27" t="n"/>
+      <c r="AL12" s="30" t="n"/>
+      <c r="AM12" s="30" t="n"/>
+      <c r="AN12" s="30" t="n"/>
+      <c r="AO12" s="30" t="n"/>
+      <c r="AP12" s="30" t="n"/>
+      <c r="AQ12" s="30" t="n"/>
+      <c r="AR12" s="30" t="n"/>
+    </row>
+    <row r="13" ht="36" customHeight="1">
+      <c r="A13" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C13" s="18" t="inlineStr">
+        <is>
+          <t>Обратная засыпка и уплотнение траншеи (Ку ≥ 0,95)</t>
+        </is>
+      </c>
+      <c r="D13" s="19" t="inlineStr">
+        <is>
+          <t>4(НН+80); 5(НН+25)</t>
+        </is>
+      </c>
+      <c r="E13" s="19" t="inlineStr">
+        <is>
+          <t>Бр.№2 земл.</t>
+        </is>
+      </c>
+      <c r="F13" s="17" t="inlineStr">
+        <is>
+          <t>15.10.2026</t>
+        </is>
+      </c>
+      <c r="G13" s="17" t="inlineStr">
+        <is>
+          <t>01.02.2027</t>
+        </is>
+      </c>
+      <c r="H13" s="17" t="n">
+        <v>110</v>
+      </c>
+      <c r="I13" s="17" t="inlineStr">
+        <is>
+          <t>0 ★</t>
+        </is>
+      </c>
+      <c r="J13" s="22" t="n"/>
+      <c r="K13" s="22" t="n"/>
+      <c r="L13" s="22" t="n"/>
+      <c r="M13" s="22" t="n"/>
+      <c r="N13" s="22" t="n"/>
+      <c r="O13" s="22" t="n"/>
+      <c r="P13" s="22" t="n"/>
+      <c r="Q13" s="22" t="n"/>
+      <c r="R13" s="22" t="n"/>
+      <c r="S13" s="22" t="n"/>
+      <c r="T13" s="22" t="n"/>
+      <c r="U13" s="22" t="n"/>
+      <c r="V13" s="22" t="n"/>
+      <c r="W13" s="22" t="n"/>
+      <c r="X13" s="22" t="n"/>
+      <c r="Y13" s="20" t="inlineStr">
+        <is>
+          <t>★10</t>
+        </is>
+      </c>
+      <c r="Z13" s="21" t="n"/>
+      <c r="AA13" s="21" t="n"/>
+      <c r="AB13" s="21" t="n"/>
+      <c r="AC13" s="21" t="n"/>
+      <c r="AD13" s="21" t="n"/>
+      <c r="AE13" s="21" t="n"/>
+      <c r="AF13" s="21" t="n"/>
+      <c r="AG13" s="21" t="n"/>
+      <c r="AH13" s="21" t="n"/>
+      <c r="AI13" s="21" t="n"/>
+      <c r="AJ13" s="21" t="n"/>
+      <c r="AK13" s="21" t="n"/>
+      <c r="AL13" s="21" t="n"/>
+      <c r="AM13" s="21" t="n"/>
+      <c r="AN13" s="21" t="n"/>
+      <c r="AO13" s="21" t="n"/>
+      <c r="AP13" s="22" t="n"/>
+      <c r="AQ13" s="22" t="n"/>
+      <c r="AR13" s="22" t="n"/>
+    </row>
+    <row r="14" ht="36" customHeight="1">
+      <c r="A14" s="17" t="n">
+        <v>11</v>
+      </c>
+      <c r="B14" s="17" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="C14" s="18" t="inlineStr">
+        <is>
+          <t>Гидравлические испытания на прочность и герметичность</t>
+        </is>
+      </c>
+      <c r="D14" s="19" t="inlineStr">
+        <is>
+          <t>10(НН+85)</t>
+        </is>
+      </c>
+      <c r="E14" s="19" t="inlineStr">
+        <is>
+          <t>Бр.№6 исп.</t>
+        </is>
+      </c>
+      <c r="F14" s="17" t="inlineStr">
+        <is>
+          <t>08.01.2027</t>
+        </is>
+      </c>
+      <c r="G14" s="17" t="inlineStr">
+        <is>
+          <t>27.01.2027</t>
+        </is>
+      </c>
+      <c r="H14" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="I14" s="17" t="inlineStr">
+        <is>
+          <t>0 ★</t>
+        </is>
+      </c>
+      <c r="J14" s="22" t="n"/>
+      <c r="K14" s="22" t="n"/>
+      <c r="L14" s="22" t="n"/>
+      <c r="M14" s="22" t="n"/>
+      <c r="N14" s="22" t="n"/>
+      <c r="O14" s="22" t="n"/>
+      <c r="P14" s="22" t="n"/>
+      <c r="Q14" s="22" t="n"/>
+      <c r="R14" s="22" t="n"/>
+      <c r="S14" s="22" t="n"/>
+      <c r="T14" s="22" t="n"/>
+      <c r="U14" s="22" t="n"/>
+      <c r="V14" s="22" t="n"/>
+      <c r="W14" s="22" t="n"/>
+      <c r="X14" s="22" t="n"/>
+      <c r="Y14" s="22" t="n"/>
+      <c r="Z14" s="22" t="n"/>
+      <c r="AA14" s="22" t="n"/>
+      <c r="AB14" s="22" t="n"/>
+      <c r="AC14" s="22" t="n"/>
+      <c r="AD14" s="22" t="n"/>
+      <c r="AE14" s="22" t="n"/>
+      <c r="AF14" s="22" t="n"/>
+      <c r="AG14" s="22" t="n"/>
+      <c r="AH14" s="22" t="n"/>
+      <c r="AI14" s="22" t="n"/>
+      <c r="AJ14" s="22" t="n"/>
+      <c r="AK14" s="20" t="inlineStr">
+        <is>
+          <t>★11</t>
+        </is>
+      </c>
+      <c r="AL14" s="21" t="n"/>
+      <c r="AM14" s="21" t="n"/>
+      <c r="AN14" s="21" t="n"/>
+      <c r="AO14" s="22" t="n"/>
+      <c r="AP14" s="22" t="n"/>
+      <c r="AQ14" s="22" t="n"/>
+      <c r="AR14" s="22" t="n"/>
+    </row>
+    <row r="15" ht="36" customHeight="1">
+      <c r="A15" s="17" t="n">
+        <v>12</v>
+      </c>
+      <c r="B15" s="17" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="C15" s="18" t="inlineStr">
+        <is>
+          <t>Пусконаладочные работы, промывка, дезинфекция</t>
+        </is>
+      </c>
+      <c r="D15" s="19" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="E15" s="19" t="inlineStr">
+        <is>
+          <t>Бр.№6 ПНР</t>
+        </is>
+      </c>
+      <c r="F15" s="17" t="inlineStr">
+        <is>
+          <t>28.01.2027</t>
+        </is>
+      </c>
+      <c r="G15" s="17" t="inlineStr">
+        <is>
+          <t>11.02.2027</t>
+        </is>
+      </c>
+      <c r="H15" s="17" t="n">
+        <v>15</v>
+      </c>
+      <c r="I15" s="17" t="inlineStr">
+        <is>
+          <t>0 ★</t>
+        </is>
+      </c>
+      <c r="J15" s="22" t="n"/>
+      <c r="K15" s="22" t="n"/>
+      <c r="L15" s="22" t="n"/>
+      <c r="M15" s="22" t="n"/>
+      <c r="N15" s="22" t="n"/>
+      <c r="O15" s="22" t="n"/>
+      <c r="P15" s="22" t="n"/>
+      <c r="Q15" s="22" t="n"/>
+      <c r="R15" s="22" t="n"/>
+      <c r="S15" s="22" t="n"/>
+      <c r="T15" s="22" t="n"/>
+      <c r="U15" s="22" t="n"/>
+      <c r="V15" s="22" t="n"/>
+      <c r="W15" s="22" t="n"/>
+      <c r="X15" s="22" t="n"/>
+      <c r="Y15" s="22" t="n"/>
+      <c r="Z15" s="22" t="n"/>
+      <c r="AA15" s="22" t="n"/>
+      <c r="AB15" s="22" t="n"/>
+      <c r="AC15" s="22" t="n"/>
+      <c r="AD15" s="22" t="n"/>
+      <c r="AE15" s="22" t="n"/>
+      <c r="AF15" s="22" t="n"/>
+      <c r="AG15" s="22" t="n"/>
+      <c r="AH15" s="22" t="n"/>
+      <c r="AI15" s="22" t="n"/>
+      <c r="AJ15" s="22" t="n"/>
+      <c r="AK15" s="22" t="n"/>
+      <c r="AL15" s="22" t="n"/>
+      <c r="AM15" s="22" t="n"/>
+      <c r="AN15" s="20" t="inlineStr">
+        <is>
+          <t>★12</t>
+        </is>
+      </c>
+      <c r="AO15" s="21" t="n"/>
+      <c r="AP15" s="21" t="n"/>
+      <c r="AQ15" s="22" t="n"/>
+      <c r="AR15" s="22" t="n"/>
+    </row>
+    <row r="16" ht="36" customHeight="1">
+      <c r="A16" s="28" t="n">
+        <v>13</v>
+      </c>
+      <c r="B16" s="28" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="C16" s="29" t="inlineStr">
+        <is>
+          <t>Благоустройство и рекультивация, восстановление покрытий</t>
+        </is>
+      </c>
+      <c r="D16" s="29" t="inlineStr">
+        <is>
+          <t>10(НН+30)</t>
+        </is>
+      </c>
+      <c r="E16" s="29" t="inlineStr">
+        <is>
+          <t>Бр.№7 благ.</t>
+        </is>
+      </c>
+      <c r="F16" s="28" t="inlineStr">
+        <is>
+          <t>14.11.2026</t>
+        </is>
+      </c>
+      <c r="G16" s="28" t="inlineStr">
+        <is>
+          <t>16.02.2027</t>
+        </is>
+      </c>
+      <c r="H16" s="28" t="n">
+        <v>95</v>
+      </c>
+      <c r="I16" s="28" t="n">
+        <v>5</v>
+      </c>
+      <c r="J16" s="30" t="n"/>
+      <c r="K16" s="30" t="n"/>
+      <c r="L16" s="30" t="n"/>
+      <c r="M16" s="30" t="n"/>
+      <c r="N16" s="30" t="n"/>
+      <c r="O16" s="30" t="n"/>
+      <c r="P16" s="30" t="n"/>
+      <c r="Q16" s="30" t="n"/>
+      <c r="R16" s="30" t="n"/>
+      <c r="S16" s="30" t="n"/>
+      <c r="T16" s="30" t="n"/>
+      <c r="U16" s="30" t="n"/>
+      <c r="V16" s="30" t="n"/>
+      <c r="W16" s="30" t="n"/>
+      <c r="X16" s="30" t="n"/>
+      <c r="Y16" s="30" t="n"/>
+      <c r="Z16" s="30" t="n"/>
+      <c r="AA16" s="30" t="n"/>
+      <c r="AB16" s="30" t="n"/>
+      <c r="AC16" s="30" t="n"/>
+      <c r="AD16" s="26" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="AE16" s="27" t="n"/>
+      <c r="AF16" s="27" t="n"/>
+      <c r="AG16" s="27" t="n"/>
+      <c r="AH16" s="27" t="n"/>
+      <c r="AI16" s="27" t="n"/>
+      <c r="AJ16" s="27" t="n"/>
+      <c r="AK16" s="27" t="n"/>
+      <c r="AL16" s="27" t="n"/>
+      <c r="AM16" s="27" t="n"/>
+      <c r="AN16" s="27" t="n"/>
+      <c r="AO16" s="27" t="n"/>
+      <c r="AP16" s="27" t="n"/>
+      <c r="AQ16" s="27" t="n"/>
+      <c r="AR16" s="30" t="n"/>
+    </row>
+    <row r="17" ht="36" customHeight="1">
+      <c r="A17" s="17" t="n">
+        <v>14</v>
+      </c>
+      <c r="B17" s="17" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="C17" s="18" t="inlineStr">
+        <is>
+          <t>Оформление испол. документации, сдача комиссии, КС-11</t>
+        </is>
+      </c>
+      <c r="D17" s="19" t="inlineStr">
+        <is>
+          <t>12(НН+5)</t>
+        </is>
+      </c>
+      <c r="E17" s="19" t="inlineStr">
+        <is>
+          <t>ПТО + ИТР</t>
+        </is>
+      </c>
+      <c r="F17" s="17" t="inlineStr">
+        <is>
+          <t>02.02.2027</t>
+        </is>
+      </c>
+      <c r="G17" s="17" t="inlineStr">
+        <is>
+          <t>21.02.2027</t>
+        </is>
+      </c>
+      <c r="H17" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="I17" s="17" t="inlineStr">
+        <is>
+          <t>0 ★</t>
+        </is>
+      </c>
+      <c r="J17" s="22" t="n"/>
+      <c r="K17" s="22" t="n"/>
+      <c r="L17" s="22" t="n"/>
+      <c r="M17" s="22" t="n"/>
+      <c r="N17" s="22" t="n"/>
+      <c r="O17" s="22" t="n"/>
+      <c r="P17" s="22" t="n"/>
+      <c r="Q17" s="22" t="n"/>
+      <c r="R17" s="22" t="n"/>
+      <c r="S17" s="22" t="n"/>
+      <c r="T17" s="22" t="n"/>
+      <c r="U17" s="22" t="n"/>
+      <c r="V17" s="22" t="n"/>
+      <c r="W17" s="22" t="n"/>
+      <c r="X17" s="22" t="n"/>
+      <c r="Y17" s="22" t="n"/>
+      <c r="Z17" s="22" t="n"/>
+      <c r="AA17" s="22" t="n"/>
+      <c r="AB17" s="22" t="n"/>
+      <c r="AC17" s="22" t="n"/>
+      <c r="AD17" s="22" t="n"/>
+      <c r="AE17" s="22" t="n"/>
+      <c r="AF17" s="22" t="n"/>
+      <c r="AG17" s="22" t="n"/>
+      <c r="AH17" s="22" t="n"/>
+      <c r="AI17" s="22" t="n"/>
+      <c r="AJ17" s="22" t="n"/>
+      <c r="AK17" s="22" t="n"/>
+      <c r="AL17" s="22" t="n"/>
+      <c r="AM17" s="22" t="n"/>
+      <c r="AN17" s="22" t="n"/>
+      <c r="AO17" s="20" t="inlineStr">
+        <is>
+          <t>★14</t>
+        </is>
+      </c>
+      <c r="AP17" s="21" t="n"/>
+      <c r="AQ17" s="21" t="n"/>
+      <c r="AR17" s="21" t="n"/>
+    </row>
+    <row r="19" ht="34" customHeight="1">
+      <c r="A19" s="31" t="inlineStr">
+        <is>
+          <t>УСЛОВНЫЕ ОБОЗНАЧЕНИЯ:   █ критический путь (★) — красно-оранжевый;   █ работы с резервом — синий;   Предшественники: ОН — окончание‑начало, НН — начало‑начало, ОО — окончание‑окончание,  цифра — № работы,  (+X) — лаг, дн.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="32" t="inlineStr">
+        <is>
+          <t>ИТОГО по объекту: с 27.06.2026 по 21.02.2027</t>
+        </is>
+      </c>
+      <c r="H20" s="33" t="n">
+        <v>240</v>
+      </c>
+      <c r="I20" s="34" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="21">
+    <mergeCell ref="A19:AR19"/>
+    <mergeCell ref="X2:AB2"/>
+    <mergeCell ref="A20:G20"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="AC2:AF2"/>
+    <mergeCell ref="J2"/>
+    <mergeCell ref="F2:F3"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="AP2:AR2"/>
+    <mergeCell ref="A1:AR1"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="AG2:AJ2"/>
+    <mergeCell ref="O2:S2"/>
+    <mergeCell ref="T2:W2"/>
+    <mergeCell ref="K2:N2"/>
+    <mergeCell ref="AK2:AO2"/>
+    <mergeCell ref="G2:G3"/>
+    <mergeCell ref="I2:I3"/>
+  </mergeCells>
+  <printOptions gridLines="0"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="8" fitToHeight="1" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1028,6 +2738,9 @@
           <t>ИТОГО по объекту: с 27.06.2026 по 21.02.2027</t>
         </is>
       </c>
+      <c r="B17" s="35" t="n"/>
+      <c r="C17" s="35" t="n"/>
+      <c r="D17" s="36" t="n"/>
       <c r="E17" s="11" t="n">
         <v>240</v>
       </c>

</xml_diff>